<commit_message>
20260113: Update DRC for Floating Gate check.
</commit_message>
<xml_diff>
--- a/Document/TR-1um_Drawing_Layer_DR_Table.xlsx
+++ b/Document/TR-1um_Drawing_Layer_DR_Table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/okamura/Library/CloudStorage/Dropbox/91_OpenPDK/TR-1um/Document/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A87561A-1DD7-6246-981C-42DFCC05E15B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A23B3161-895D-DF4B-905C-891163F654C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="900" yWindow="760" windowWidth="29440" windowHeight="18880" xr2:uid="{7F1200E8-B51D-9446-A5CE-CEA05B5231B7}"/>
+    <workbookView xWindow="800" yWindow="760" windowWidth="29440" windowHeight="18880" xr2:uid="{7F1200E8-B51D-9446-A5CE-CEA05B5231B7}"/>
   </bookViews>
   <sheets>
     <sheet name="TR-1um_Drawing_Layer_DR_Table" sheetId="2" r:id="rId1"/>
@@ -929,12 +929,6 @@
     <t>PO.Z2</t>
   </si>
   <si>
-    <t>Electrical</t>
-  </si>
-  <si>
-    <t>ANT</t>
-  </si>
-  <si>
     <t>Prohibited</t>
   </si>
   <si>
@@ -957,6 +951,12 @@
   </si>
   <si>
     <t>CO.GG</t>
+  </si>
+  <si>
+    <t>Electrical / Optional</t>
+  </si>
+  <si>
+    <t>ANTE</t>
   </si>
 </sst>
 </file>
@@ -2050,7 +2050,7 @@
         <v>188</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="D2" s="23"/>
       <c r="E2" s="22"/>
@@ -2235,16 +2235,16 @@
     </row>
     <row r="12" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="5" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="C12" s="11" t="s">
         <v>261</v>
       </c>
       <c r="D12" s="11" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="F12" s="6">
         <v>0</v>
@@ -3446,7 +3446,7 @@
     </row>
     <row r="71" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B71" s="5" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="C71" s="11" t="s">
         <v>146</v>
@@ -3473,7 +3473,7 @@
         <v>146</v>
       </c>
       <c r="D72" s="11" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="E72" s="5" t="s">
         <v>136</v>
@@ -3594,7 +3594,7 @@
         <v>124</v>
       </c>
       <c r="C78" s="13" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="D78" s="13"/>
       <c r="E78" s="8" t="s">
@@ -3632,7 +3632,7 @@
         <v>211</v>
       </c>
       <c r="C80" s="13" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="D80" s="13" t="s">
         <v>143</v>
@@ -3656,7 +3656,7 @@
         <v>149</v>
       </c>
       <c r="D81" s="13" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="E81" s="8" t="s">
         <v>165</v>
@@ -3672,7 +3672,7 @@
         <v>218</v>
       </c>
       <c r="C82" s="13" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="D82" s="13" t="s">
         <v>159</v>
@@ -4781,7 +4781,7 @@
         <v>261</v>
       </c>
       <c r="D136" s="26" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="E136" s="25" t="s">
         <v>136</v>
@@ -4980,7 +4980,7 @@
         <v>188</v>
       </c>
       <c r="C146" s="18" t="s">
-        <v>297</v>
+        <v>305</v>
       </c>
       <c r="D146" s="23"/>
       <c r="E146" s="22"/>
@@ -5013,14 +5013,14 @@
     </row>
     <row r="148" spans="2:8" ht="20" x14ac:dyDescent="0.2">
       <c r="B148" s="25" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="C148" s="26" t="s">
-        <v>303</v>
+        <v>204</v>
       </c>
       <c r="D148" s="26"/>
       <c r="E148" s="25" t="s">
-        <v>298</v>
+        <v>306</v>
       </c>
       <c r="F148" s="28">
         <v>0</v>

</xml_diff>

<commit_message>
Add TR-1um DRC runset and CSV-to-DRC generator
- Import TR-1um rule definitions
- Add script to generate KLayout DRC runset from CSV
- Prepare initial framework for rule maintenance and automation
</commit_message>
<xml_diff>
--- a/Document/TR-1um_Drawing_Layer_DR_Table.xlsx
+++ b/Document/TR-1um_Drawing_Layer_DR_Table.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/okamura/Library/CloudStorage/Dropbox/91_OpenPDK/TR-1um/Document/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/okamura/Dropbox/91_OpenPDK/TR-1um/Document/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A23B3161-895D-DF4B-905C-891163F654C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{439FB1C9-0C98-1F41-9D86-FF4ED4B90AE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="800" yWindow="760" windowWidth="29440" windowHeight="18880" xr2:uid="{7F1200E8-B51D-9446-A5CE-CEA05B5231B7}"/>
+    <workbookView xWindow="860" yWindow="760" windowWidth="29380" windowHeight="18880" xr2:uid="{7F1200E8-B51D-9446-A5CE-CEA05B5231B7}"/>
   </bookViews>
   <sheets>
     <sheet name="TR-1um_Drawing_Layer_DR_Table" sheetId="2" r:id="rId1"/>
@@ -3205,7 +3205,7 @@
       </c>
       <c r="D59" s="13"/>
       <c r="E59" s="8" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="F59" s="9">
         <v>1</v>

</xml_diff>